<commit_message>
feat: FR-07 ижил төстэй бодлого + Supabase DB, RLS migration
- services/similar.py, POST /similar, /uploads/{id}/outcome; solution_steps (0004)
- ml/tools/bank_steps.py: 200 бодлогын алхамчилсан бодолт
- Supabase (Session pooler) тохиргоо, 0005 RLS, docker-entrypoint (alembic upgrade)
- docker-compose: localdb profile, ./ml → /ml:ro mount

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ml/бодлогын_сан.xlsx
+++ b/ml/бодлогын_сан.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Нэр_томьёо" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Бодлого'!$A$1:$O$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Бодлого'!$A$1:$P$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Сэдвүүд'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Сэдвийн_граф'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Нэр_томьёо'!$A$1:$D$33</definedName>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O201"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -454,6 +454,7 @@
     <col width="38" customWidth="1" min="13" max="13"/>
     <col width="38" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,6 +533,11 @@
           <t>sympy_шалгалт</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>бодолтын_алхам</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -603,6 +609,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Ижил суурьтай зэргийг үржүүлэхэд илтгэгч нэмэгдэнэ: $a^m \cdot a^n = a^{m+n}$. || $2^3 \cdot 2^2 = 2^{3+2} = 2^5$. || $2^5 = 32$.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -674,6 +685,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Хуваарийг ижил болгоно: 4 ба 6-ийн ХБЕХ нь 12. || $\frac{3}{4} = \frac{9}{12}$, $\frac{1}{6} = \frac{2}{12}$. || $\frac{9}{12} + \frac{2}{12} = \frac{11}{12}$.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -745,6 +761,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Хүртвэр: $3^4 \cdot 3^{-2} = 3^{4-2} = 3^2$. || Хуваах: $3^2 : 3^1 = 3^{2-1} = 3^1$. || Хариу: $3$.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -816,6 +837,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Язгуур доорхыг бүтэн квадратаар задална: $50 = 25 \cdot 2$, $18 = 9 \cdot 2$. || $\sqrt{50} = 5\sqrt{2}$, $\sqrt{18} = 3\sqrt{2}$. || $5\sqrt{2} - 3\sqrt{2} = 2\sqrt{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -887,6 +913,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Сөрөг илтгэгч урвуулна: $(\tfrac{1}{2})^{-3} = 2^3 = 8$. || $16^{1/2} = \sqrt{16} = 4$. || $8 + 4 = 12$.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -958,6 +989,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>$a^{m/n} = (\sqrt[n]{a})^m$: $27^{2/3} = (\sqrt[3]{27})^2 = 3^2 = 9$. || $8^{1/3} = \sqrt[3]{8} = 2$. || $9 - 2 = 7$.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1033,6 +1069,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Хаалт задлах: $3(x-4) = 3x - 12$. || $3x - 12 + 2x$. || Төсөөтэй гишүүд: $5x - 12$.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1108,6 +1149,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>$a$-тай гишүүд: $4a + a = 5a$. || $b$-тэй гишүүд: $-2b + 5b = 3b$. || Хариу: $5a + 3b$.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1183,6 +1229,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>$9 = 3^2$ тул энэ нь квадратуудын ялгавар. || $a^2 - b^2 = (a-b)(a+b)$, энд $a = x$, $b = 3$. || $(x-3)(x+3)$.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1258,6 +1309,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>$(a+b)^2 = a^2 + 2ab + b^2$. || $a = x$, $b = 3$: $x^2 + 2 \cdot x \cdot 3 + 3^2$. || $x^2 + 6x + 9$.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1333,6 +1389,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Үржвэр нь 6, нийлбэр нь $-5$ болох хоёр тоо хайна. || $-2$ ба $-3$: $(-2)(-3) = 6$, $-2 + (-3) = -5$. || $(x-2)(x-3)$.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1408,6 +1469,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Хүртвэрийг задална: $x^2 - 4 = (x-2)(x+2)$. || $\frac{(x-2)(x+2)}{x-2}$ — $x \ne 2$ тул $(x-2)$-оор хураана. || Хариу: $x + 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1483,6 +1549,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>5-ыг баруун тал руу шилжүүлнэ (тэмдэг солигдоно): $2x = 13 - 5$. || $2x = 8$. || $x = 8 : 2 = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1558,6 +1629,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>$x$-тэй гишүүдийг зүүн, тоонуудыг баруун тийш: $3x - 2x = 1 + 7$. || $x = 8$. || Шалгалт: $3 \cdot 8 - 7 = 17 = 2 \cdot 8 + 1$ ✓</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1633,6 +1709,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Хөндлөн үржүүлнэ: $5(x-1) = 3(x+1)$. || $5x - 5 = 3x + 3$ → $2x = 8$. || $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1708,6 +1789,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Үзэгний үнийг $x$ гэвэл дэвтэр $x + 300$. || $2(x+300) + 3x = 3600$ → $5x + 600 = 3600$. || $5x = 3000$ → $x = 600$ төгрөг.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1783,6 +1869,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр тэгшитгэлийг нэмнэ: $2x = 14$ → $x = 7$. || $x = 7$-г эхнийхэд орлуулна: $7 + y = 10$. || $y = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1858,6 +1949,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Хүүгийн насыг $x$ гэвэл аав $4x$. || 5 жилийн дараа: $4x + 5 = 3(x + 5)$ → $4x + 5 = 3x + 15$. || $x = 10$ настай.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1933,6 +2029,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>$x^2 = 16$. || Квадрат нь 16 болох тоо хоёр: $4$ ба $-4$. || $x = -4$; $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2008,6 +2109,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>$x$-ийг хаалтын өмнө гаргана: $x(x-5) = 0$. || Үржвэр 0 бол аль нэг үржигдэхүүн 0: $x = 0$ эсвэл $x - 5 = 0$. || $x = 0$; $x = 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2083,6 +2189,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>Виет: үржвэр 12, нийлбэр 7. || $3 \cdot 4 = 12$, $3 + 4 = 7$. || $x = 3$; $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2158,6 +2269,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>$D = b^2 - 4ac = 9 + 16 = 25$, $\sqrt{D} = 5$. || $x = \frac{-3 \pm 5}{2 \cdot 2}$. || $x_1 = \frac{2}{4} = \frac{1}{2}$, $x_2 = \frac{-8}{4} = -2$.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2233,6 +2349,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>$D = 4 + 4 = 8$, $\sqrt{8} = 2\sqrt{2}$. || $x = \frac{2 \pm 2\sqrt{2}}{2}$. || $x = 1 \pm \sqrt{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2308,6 +2429,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Давхар язгуур ⇔ $D = 0$. || $D = k^2 - 4 \cdot 9 = k^2 - 36 = 0$. || $k = \pm 6$.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2383,6 +2509,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>$2x &gt; 5 + 3$. || $2x &gt; 8$. || $x &gt; 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2458,6 +2589,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>$-3x \le -6$. || Сөрөг тоонд хуваахад тэмдэг эргэнэ. || $x \ge 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2533,6 +2669,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 4-өөр үржүүлнэ: $2(x-1) &lt; x + 3$. || $2x - 2 &lt; x + 3$ → $x &lt; 5$. || Хариу: $x &lt; 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2608,6 +2749,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>$|t| &lt; a$ ⇔ $-a &lt; t &lt; a$. || $-3 &lt; x - 2 &lt; 3$. || $-1 &lt; x &lt; 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2683,6 +2829,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>Язгуурууд: $x^2 - 5x + 6 = (x-2)(x-3)$ → $2$ ба $3$. || Дээш харсан парабол язгууруудын хооронд сөрөг. || $2 &lt; x &lt; 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2758,6 +2909,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>$(x-2)(x+2) \ge 0$, язгуурууд $\pm 2$. || Дээш харсан парабол язгууруудын гадна эерэг. || $x \le -2$ эсвэл $x \ge 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2833,6 +2989,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>$x$-ийн оронд 4 орлуулна: $f(4) = 3 \cdot 4 - 2$. || $12 - 2$. || $f(4) = 10$.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2908,6 +3069,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>$y = kx + b$ хэлбэрт $k$ нь өнцгийн коэффициент. || $y = 2x + 1$ → $k = 2$, $b = 1$. || Хариу: $2$.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2983,6 +3149,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>Язгуур доорх илэрхийлэл сөрөг биш байх ёстой: $x - 3 \ge 0$. || $x \ge 3$. || Тодорхойлогдох муж: $[3; +\infty)$.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3058,6 +3229,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>$k = \frac{y_2 - y_1}{x_2 - x_1} = \frac{7-3}{3-1} = 2$. || $y = 2x + b$-д $(1;3)$ орлуулна: $3 = 2 + b$ → $b = 1$. || $y = 2x + 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3133,6 +3309,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>Оройн абсцисс $x_0 = -\frac{b}{2a} = \frac{4}{2} = 2$. || $y_0 = f(2) = 4 - 8 + 1 = -3$. || Орой: $(2; -3)$.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3208,6 +3389,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P37" s="2" t="inlineStr">
+        <is>
+          <t>Дотоод функц эхлээд: $g(2) = 2^2 = 4$. || $f(4) = 2 \cdot 4 + 3$. || $f(g(2)) = 11$.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3283,6 +3469,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>$8 = 2^3$. || $2^x = 2^3$ → суурь ижил тул илтгэгчүүд тэнцүү. || $x = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3358,6 +3549,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>$\frac{1}{9} = 3^{-2}$. || $3^x = 3^{-2}$. || $x = -2$.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3433,6 +3629,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>$4 = 2^2$, $32 = 2^5$. || $(2^2)^x = 2^5$ → $2^{2x} = 2^5$. || $2x = 5$ → $x = \frac{5}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3508,6 +3709,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>$125 = 5^3$. || $5^{x+1} = 5^3$ → $x + 1 = 3$. || $x = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3583,6 +3789,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>$t = 2^x$ ($t &gt; 0$): $t^2 - 3t - 4 = 0$. || $t = 4$ эсвэл $t = -1$ (тохирохгүй). || $2^x = 4$ → $x = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3658,6 +3869,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>$9^x = (3^x)^2$, $t = 3^x$: $t^2 - 4t + 3 = 0$. || $t = 1$ эсвэл $t = 3$. || $3^x = 1$ → $x = 0$; $3^x = 3$ → $x = 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3733,6 +3949,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>$\log_2 16$: 2-ыг хэдэн зэрэгт дэвшүүлбэл 16? || $2^4 = 16$. || Хариу: $4$.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3808,6 +4029,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>$\lg$ = 10 суурьтай логарифм. || $10^3 = 1000$. || $\lg 1000 = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3883,6 +4109,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>$\log_3 27 = 3$ ($3^3 = 27$). || $\log_3 \frac{1}{3} = -1$ ($3^{-1} = \frac{1}{3}$). || $3 + (-1) = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3958,6 +4189,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>Тодорхойлолт: $x - 1 = 2^3$. || $x - 1 = 8$. || $x = 9$ (шалгалт: $9 - 1 = 8 &gt; 0$ ✓).</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4033,6 +4269,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>ТМ: $x &gt; 2$. $\log_2 [x(x-2)] = 3$. || $x(x-2) = 8$ → $x^2 - 2x - 8 = 0$ → $x = 4$, $x = -2$. || $x = -2$ ТМ-д орохгүй → $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4108,6 +4349,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>$\log_a b - \log_a c = \log_a \frac{b}{c}$. || $\log_5 \frac{50}{2} = \log_5 25$. || $5^2 = 25$ → $2$.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4183,6 +4429,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>$30°$ тусгай өнцөг. || Хүснэгт: $\sin 30° = \frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4258,6 +4509,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>$\cos 60° = \frac{1}{2}$. || $\sin 90° = 1$. || $\frac{1}{2} + 1 = \frac{3}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4333,6 +4589,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>$\sin^2\alpha + \cos^2\alpha = 1$ → $\cos^2\alpha = 1 - \frac{9}{25} = \frac{16}{25}$. || Хурц өнцөгт $\cos\alpha &gt; 0$. || $\cos\alpha = \frac{4}{5}$.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4408,6 +4669,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>$\operatorname{tg}45° = 1$, $\cos 0° = 1$, $\sin 30° = \frac{1}{2}$. || $1 \cdot 1 - (\tfrac{1}{2})^2 = 1 - \frac{1}{4}$. || $\frac{3}{4}$.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4483,6 +4749,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>Нэгж тойрог дээр $\sin x = \frac{1}{2}$: I мөчлөгт $x = \frac{\pi}{6}$. || II мөчлөгт $x = \pi - \frac{\pi}{6} = \frac{5\pi}{6}$. || $x = \frac{\pi}{6}$; $x = \frac{5\pi}{6}$.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4558,6 +4829,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>$1 - \cos^2\alpha = \sin^2\alpha$. || $\frac{\sin^2\alpha}{\sin\alpha}$. || $\sin\alpha$.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4633,6 +4909,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>Боломжит үр дүн: 1, 2, 3, 4, 5, 6 — нийт 6. || Тэгш: 2, 4, 6 — 3 ширхэг. || $P = \frac{3}{6} = \frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4708,6 +4989,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Нийт бөмбөг: $3 + 5 = 8$. || Таатай (улаан): 3. || $P = \frac{3}{8}$.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4783,6 +5069,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>5 хүний сэлгэмэл: $P_5 = 5!$. || $5 \cdot 4 \cdot 3 \cdot 2 \cdot 1$. || $120$.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4858,6 +5149,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
+          <t>Дараалал чухал биш → хэсэглэл $C_8^3 = \frac{8!}{3! \cdot 5!}$. || $\frac{8 \cdot 7 \cdot 6}{3 \cdot 2 \cdot 1} = \frac{336}{6}$. || $56$.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4933,6 +5229,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Нийт үр дүн $6 \cdot 6 = 36$. || Нийлбэр 7: (1,6),(2,5),(3,4),(4,3),(5,2),(6,1) — 6 хос. || $P = \frac{6}{36} = \frac{1}{6}$.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5008,6 +5309,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Нийт үр дүн $2^3 = 8$. || Яг 2 сүлд: ССТ, СТС, ТСС — $C_3^2 = 3$. || $P = \frac{3}{8}$.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5079,6 +5385,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>$5 = 5^1$ гэж бичнэ. || $5^2 \cdot 5^1 = 5^{2+1} = 5^3$. || $5^3 = 125$.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5150,6 +5461,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Ижил суурьтай зэргийг хуваахад илтгэгч хасагдана: $a^m : a^n = a^{m-n}$. || $7^{5-3} = 7^2$. || $7^2 = 49$.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5221,6 +5537,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>Үйлдлийн дараалал: эхлээд зэрэг $4^2 = 16$. || Дараа нь үржих: $2 \cdot 16 = 32$. || Сүүлд нэмэх: $3 + 32 = 35$.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5292,6 +5613,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Үржүүлэхээс өмнө хураана: 2 ба 4-ийг 2-т, 3 ба 9-ийг 3-т. || $\frac{1}{1} \cdot \frac{3}{2}$. || Хариу: $\frac{3}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5363,6 +5689,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>ХБЕХ(6, 4) = 12. || $\frac{5}{6} = \frac{10}{12}$, $\frac{1}{4} = \frac{3}{12}$. || $\frac{10}{12} - \frac{3}{12} = \frac{7}{12}$.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5434,6 +5765,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>Зэргийн зэрэг: $(a^m)^n = a^{mn}$, тэгэхээр $(2^3)^2 = 2^6$. || $2^6 : 2^4 = 2^{6-4} = 2^2$. || $2^2 = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5505,6 +5841,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>$2^{-3} = \frac{1}{2^3} = \frac{1}{8}$. || $4^{-1} = \frac{1}{4} = \frac{2}{8}$. || $\frac{1}{8} + \frac{2}{8} = \frac{3}{8}$.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5576,6 +5917,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>$12 = 4 \cdot 3$, $27 = 9 \cdot 3$. || $\sqrt{12} = 2\sqrt{3}$, $\sqrt{27} = 3\sqrt{3}$. || $2\sqrt{3} + 3\sqrt{3} = 5\sqrt{3}$.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5647,6 +5993,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>$\sqrt{a} \cdot \sqrt{b} = \sqrt{ab}$. || $\sqrt{3 \cdot 12} = \sqrt{36}$. || $\sqrt{36} = 6$.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5718,6 +6069,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>Тоонуудыг тусад нь: $3 \cdot 2 = 6$. || 10-ын зэргүүдийг тусад нь: $10^4 \cdot 10^{-2} = 10^2$. || $6 \cdot 10^2 = 600$.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5789,6 +6145,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>$32 = 2^5$ тул $32^{2/5} = (2^5)^{2/5} = 2^2 = 4$. || $9^{-1/2} = \frac{1}{\sqrt{9}} = \frac{1}{3}$. || $4 + \frac{1}{3} = \frac{13}{3}$.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5860,6 +6221,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>$6^5 = (2 \cdot 3)^5 = 2^5 \cdot 3^5$. || $\frac{2^5 \cdot 3^5}{2^5 \cdot 3^3} = 3^{5-3}$. || $3^2 = 9$.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5931,6 +6297,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>$(a-b)(a+b) = a^2 - b^2$ томьёо. || $(\sqrt{5})^2 - 1^2 = 5 - 1$. || Хариу: $4$.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -6002,6 +6373,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P75" s="2" t="inlineStr">
+        <is>
+          <t>Анхны үнийг $x$ гэвэл 20% нэмэгдсэн үнэ $1{,}2x$. || $1{,}2x = 24000$. || $x = 24000 : 1{,}2 = 20000$ төгрөг.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -6077,6 +6453,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>$2(3x+1) = 6x + 2$. || $6x + 2 - 4x$. || $2x + 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -6152,6 +6533,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>Хаалтын өмнөх хасах тэмдэг гишүүн бүрийн тэмдгийг солино: $-(x-5) = -x + 5$. || $-x + 5 + 3x$. || $2x + 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -6227,6 +6613,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>$x^2$-тэй гишүүд: $3x^2 - x^2 = 2x^2$. || $x$-тэй гишүүд: $2x + 4x = 6x$. || $2x^2 + 6x$ ($x^2$ ба $x$ нэгтгэгдэхгүй).</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6302,6 +6693,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>Коэффициентуудын ЕХ: $6$ ба $9$ → $3$; $x^2$ ба $x$ → $x$. || Ерөнхий үржигдэхүүн $3x$. || $6x^2 : 3x = 2x$, $9x : 3x = 3$ → $3x(2x+3)$.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -6377,6 +6773,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>$x = -2$-ыг хаалттай орлуулна: $(-2)^2 - 3(-2) + 1$. || $(-2)^2 = 4$, $-3 \cdot (-2) = +6$. || $4 + 6 + 1 = 11$.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -6452,6 +6853,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P81" s="2" t="inlineStr">
+        <is>
+          <t>$(a-b)^2 = a^2 - 2ab + b^2$, $a = 2x$, $b = 1$. || $(2x)^2 - 2 \cdot 2x \cdot 1 + 1^2$. || $4x^2 - 4x + 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -6527,6 +6933,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>$(a-b)(a+b) = a^2 - b^2$. || $a = x$, $b = 4$. || $x^2 - 16$.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6602,6 +7013,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P83" s="2" t="inlineStr">
+        <is>
+          <t>$4x^2 = (2x)^2$, $25 = 5^2$. || Квадратуудын ялгавар: $(2x)^2 - 5^2$. || $(2x-5)(2x+5)$.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6677,6 +7093,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>Үржвэр 10, нийлбэр 7 болох хоёр тоо. || $2 \cdot 5 = 10$, $2 + 5 = 7$. || $(x+2)(x+5)$.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6752,6 +7173,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P85" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр хоёроор бүлэглэнэ: $(x^2 + 3x) + (xy + 3y)$. || $x(x+3) + y(x+3)$. || Ерөнхий хаалт: $(x+3)(x+y)$.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6827,6 +7253,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P86" s="2" t="inlineStr">
+        <is>
+          <t>Хүртвэр бүтэн квадрат: $x^2 + 6x + 9 = (x+3)^2$. || $\frac{(x+3)^2}{x+3}$, $x \ne -3$. || $x + 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6902,6 +7333,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P87" s="2" t="inlineStr">
+        <is>
+          <t>Ерөнхий хуваарь $x(x+1)$. || $\frac{x+1}{x(x+1)} + \frac{x}{x(x+1)}$. || $\frac{2x+1}{x(x+1)}$.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6977,6 +7413,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P88" s="2" t="inlineStr">
+        <is>
+          <t>$(a+b)^3 = a^3 + 3a^2b + 3ab^2 + b^3$. || $a = x$, $b = 2$: $x^3 + 3x^2 \cdot 2 + 3x \cdot 4 + 8$. || $x^3 + 6x^2 + 12x + 8$.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -7052,6 +7493,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P89" s="2" t="inlineStr">
+        <is>
+          <t>$x^2 - 6x$ нь $(x-3)^2 = x^2 - 6x + 9$-ийн эхлэл. || $x^2 - 6x + 13 = (x-3)^2 - 9 + 13$. || $= (x-3)^2 + 4$, тэгэхээр $b = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -7127,6 +7573,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>$5x = 12 + 3$. || $5x = 15$. || $x = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -7202,6 +7653,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P91" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 4-өөр үржүүлнэ. || $x = 6 \cdot 4$. || $x = 24$.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7277,6 +7733,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>$-2x = 1 - 7$. || $-2x = -6$. || $x = -6 : (-2) = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -7352,6 +7813,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P93" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 3-т хуваана: $x - 2 = 3$. || $x = 3 + 2$. || $x = 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -7427,6 +7893,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>Хаалт задлах: $2x + 6 = 5x - 6$. || $6 + 6 = 5x - 2x$ → $12 = 3x$. || $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -7502,6 +7973,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P95" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 6-аар үржүүлнэ: $3x + 2x = 30$. || $5x = 30$. || $x = 6$.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7577,6 +8053,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P96" s="2" t="inlineStr">
+        <is>
+          <t>Хөндлөн үржүүлнэ: $3 \cdot 12 = 9x$. || $36 = 9x$. || $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -7652,6 +8133,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P97" s="2" t="inlineStr">
+        <is>
+          <t>Бага тоог $x$ гэвэл $x,\ x+1,\ x+2$. || $3x + 3 = 48$ → $3x = 45$. || $x = 15$.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7727,6 +8213,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P98" s="2" t="inlineStr">
+        <is>
+          <t>Нэмнэ: $2x = 8$ → $x = 4$. || $4 + y = 7$. || $y = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7802,6 +8293,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P99" s="2" t="inlineStr">
+        <is>
+          <t>$y$-ийн коэффициентууд $+1$, $-1$ — нэмнэ: $3x = 9$ → $x = 3$. || $3 - y = 1$. || $y = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7877,6 +8373,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>$x = 2y$-г орлуулна: $3(2y) + 2y = 12$. || $8y = 12$ → $y = \frac{3}{2}$. || $x = 2 \cdot \frac{3}{2} = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7952,6 +8453,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P101" s="2" t="inlineStr">
+        <is>
+          <t>Бага тоо $x$, их тоо $x + 8$. || $x + x + 8 = 30$ → $2x = 22$. || $x = 11$.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -8027,6 +8533,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P102" s="2" t="inlineStr">
+        <is>
+          <t>Эхний хэсгийн зам: $60 \cdot 2 = 120$ км. || Үлдсэн зам: $280 - 120 = 160$ км, $80t = 160$. || $t = 2$ цаг.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -8102,6 +8613,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P103" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 2-оор үржүүлнэ: $x + 3 = 4x - 6$. || $3 + 6 = 4x - x$ → $9 = 3x$. || $x = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8177,6 +8693,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P104" s="2" t="inlineStr">
+        <is>
+          <t>Квадрат нь 49 болох тоо. || $7^2 = 49$ ба $(-7)^2 = 49$. || $x = \pm 7$.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8252,6 +8773,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P105" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 3-т хуваана: $x^2 - 9 = 0$. || $x^2 = 9$. || $x = \pm 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -8327,6 +8853,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P106" s="2" t="inlineStr">
+        <is>
+          <t>$x(x+4) = 0$. || $x = 0$ эсвэл $x + 4 = 0$. || $x = -4$; $x = 0$.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -8402,6 +8933,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P107" s="2" t="inlineStr">
+        <is>
+          <t>Үржвэр 6, нийлбэр 5. || $2 \cdot 3 = 6$, $2 + 3 = 5$. || $x = 2$; $x = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -8477,6 +9013,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P108" s="2" t="inlineStr">
+        <is>
+          <t>Үржвэр $-15$, нийлбэр $-2$. || $-5 \cdot 3 = -15$, $-5 + 3 = -2$ → $(x+5)(x-3) = 0$. || $x = -5$; $x = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -8552,6 +9093,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P109" s="2" t="inlineStr">
+        <is>
+          <t>$D = 36 - 36 = 0$ → ганц (давхар) язгуур. || $x = \frac{-b}{2a} = \frac{6}{2}$. || $x = 3$ (мөн $(x-3)^2 = 0$).</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8627,6 +9173,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P110" s="2" t="inlineStr">
+        <is>
+          <t>$D = 25 - 16 = 9$, $\sqrt{D} = 3$. || $x = \frac{5 \pm 3}{4}$. || $x_1 = 2$, $x_2 = \frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8702,6 +9253,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P111" s="2" t="inlineStr">
+        <is>
+          <t>$D = b^2 - 4ac = 9 - 20 = -11$. || $D &lt; 0$ бол бодит шийд байхгүй. || Хариу: 0 шийдтэй.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8777,6 +9333,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P112" s="2" t="inlineStr">
+        <is>
+          <t>Өргөн $x$, урт $x + 3$: $x(x+3) = 40$. || $x^2 + 3x - 40 = 0$ → үржвэр $-40$, нийлбэр 3: $8$ ба $-5$. || $x = 5$ ($x = -8$ урт байж болохгүй).</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8852,6 +9413,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P113" s="2" t="inlineStr">
+        <is>
+          <t>$D = 16 - 4 = 12$, $\sqrt{12} = 2\sqrt{3}$. || $x = \frac{-4 \pm 2\sqrt{3}}{2}$. || $x = -2 \pm \sqrt{3}$.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8927,6 +9493,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P114" s="2" t="inlineStr">
+        <is>
+          <t>Язгуур $x = 2$-ыг орлуулна: $4 - 16 + c = 0$. || $-12 + c = 0$. || $c = 12$.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9002,6 +9573,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P115" s="2" t="inlineStr">
+        <is>
+          <t>Виет: $x_1 + x_2 = 7$, $x_1 x_2 = 10$. || $x_1^2 + x_2^2 = (x_1+x_2)^2 - 2x_1x_2$. || $49 - 20 = 29$.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -9077,6 +9653,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P116" s="2" t="inlineStr">
+        <is>
+          <t>$t = x^2$: $t^2 - 5t + 4 = 0$ → $t = 1$, $t = 4$. || $x^2 = 1$ → $x = \pm 1$; $x^2 = 4$ → $x = \pm 2$. || $x = -2; -1; 1; 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -9152,6 +9733,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>$x(x+1) = 72$ → $x^2 + x - 72 = 0$. || Үржвэр $-72$, нийлбэр 1: $9$ ба $-8$. || $x = 8$ (натурал тоо).</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -9227,6 +9813,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>$x &lt; 9 - 4$. || Тэмдэг хэвээр. || $x &lt; 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9302,6 +9893,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг 3-т хуваана (эерэг — тэмдэг хэвээр). || $x \ge 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -9377,6 +9973,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр талыг $-2$-т хуваана. || Сөрөг тоонд хуваахад тэмдэг эргэнэ: $x &lt; -4$.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -9452,6 +10053,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P121" s="2" t="inlineStr">
+        <is>
+          <t>$-x \le 2 - 5 = -3$. || $-1$-ээр үржүүлж тэмдэг эргүүлнэ. || $x \ge 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9527,6 +10133,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P122" s="2" t="inlineStr">
+        <is>
+          <t>$2x - 2 &gt; x + 3$. || $2x - x &gt; 3 + 2$. || $x &gt; 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -9602,6 +10213,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P123" s="2" t="inlineStr">
+        <is>
+          <t>Гурван хэсгээс 3 хасна: $-4 \le 2x &lt; 4$. || Гурван хэсгийг 2-т хуваана. || $-2 \le x &lt; 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -9677,6 +10293,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>$|x| \le 3$ гэдэг нь $x$ нь $-3$ ба $3$-ын хооронд. || $-3 \le x \le 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -9752,6 +10373,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P125" s="2" t="inlineStr">
+        <is>
+          <t>$|t| &gt; a$ ⇔ $t &lt; -a$ эсвэл $t &gt; a$. || $x + 1 &lt; -2$ эсвэл $x + 1 &gt; 2$. || $x &lt; -3$ эсвэл $x &gt; 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9827,6 +10453,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр нөхцөл зэрэг биелэх ёстой — огтлолцол. || $x &gt; 1$ ба $x \le 4$. || $1 &lt; x \le 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -9902,6 +10533,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P127" s="2" t="inlineStr">
+        <is>
+          <t>$(x-3)(x+3) &lt; 0$, язгуурууд $\pm 3$. || Язгууруудын хооронд сөрөг. || $-3 &lt; x &lt; 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9977,6 +10613,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P128" s="2" t="inlineStr">
+        <is>
+          <t>Язгуурууд: $x^2 + x - 6 = (x+3)(x-2)$ → $-3$, $2$. || Дээш харсан парабол, $\ge 0$ гадна талд. || $x \le -3$ эсвэл $x \ge 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -10052,6 +10693,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P129" s="2" t="inlineStr">
+        <is>
+          <t>Чухал цэгүүд: $x = 2$ (хүртвэр 0), $x = -1$ (хуваарь 0, оруулахгүй). || Мужууд: $x &lt; -1$: $\frac{-}{-} &gt; 0$ ✓; $-1 &lt; x &lt; 2$: $\frac{-}{+} &lt; 0$; $x &gt; 2$: $\frac{+}{+} &gt; 0$ ✓. || $x &lt; -1$ эсвэл $x &gt; 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -10127,6 +10773,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P130" s="2" t="inlineStr">
+        <is>
+          <t>$1000 + 800x \le 9000$. || $800x \le 8000$. || $x \le 10$ → дээд тал нь 10 км.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -10202,6 +10853,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P131" s="2" t="inlineStr">
+        <is>
+          <t>Квадрат үргэлж $\ge 0$, зөвхөн $x - 1 = 0$ үед 0. || $x = 1$-ээс бусад бүх $x$-д $&gt; 0$. || $x \ne 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -10277,6 +10933,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P132" s="2" t="inlineStr">
+        <is>
+          <t>$f(-3) = (-3)^2 + 1$. || $(-3)^2 = 9$. || $9 + 1 = 10$.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -10352,6 +11013,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P133" s="2" t="inlineStr">
+        <is>
+          <t>$f(x) = 1$ гэдэг нь $5 - 2x = 1$. || $-2x = -4$. || $x = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -10427,6 +11093,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P134" s="2" t="inlineStr">
+        <is>
+          <t>$Oy$ тэнхлэг дээр $x = 0$. || $y = -3 \cdot 0 + 4$. || $y = 4$ → цэг $(0; 4)$.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -10502,6 +11173,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P135" s="2" t="inlineStr">
+        <is>
+          <t>$Ox$ тэнхлэг дээр $y = 0$. || $2x - 6 = 0$. || $x = 3$ → цэг $(3; 0)$.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -10577,6 +11253,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P136" s="2" t="inlineStr">
+        <is>
+          <t>$k = \frac{y_2 - y_1}{x_2 - x_1}$. || $\frac{7 - 1}{2 - 0} = \frac{6}{2}$. || $k = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -10652,6 +11333,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P137" s="2" t="inlineStr">
+        <is>
+          <t>Хуваарь 0 байж болохгүй. || $x - 4 = 0$ → $x = 4$. || $x = 4$ мужид орохгүй.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -10727,6 +11413,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P138" s="2" t="inlineStr">
+        <is>
+          <t>$6 - 2x \ge 0$. || $-2x \ge -6$ → тэмдэг эргэнэ. || $x \le 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10802,6 +11493,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P139" s="2" t="inlineStr">
+        <is>
+          <t>$Ox$ дээр $y = 0$: $x^2 - 2x - 3 = 0$. || Үржвэр $-3$, нийлбэр 2: $3$ ба $-1$. || $x = -1$; $x = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10877,6 +11573,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P140" s="2" t="inlineStr">
+        <is>
+          <t>$x_0 = -\frac{b}{2a}$, $a = 1$, $b = -6$. || $x_0 = \frac{6}{2}$. || $x_0 = 3$.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -10952,6 +11653,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P141" s="2" t="inlineStr">
+        <is>
+          <t>Шугаман функц $y = kx + b$: $k &gt; 0$ өснө, $k &lt; 0$ буурна. || $k = -2 &lt; 0$. || Буурна → $-1$.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -11027,6 +11733,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P142" s="2" t="inlineStr">
+        <is>
+          <t>$a = -1 &lt; 0$ тул парабол доош харсан, оройд хамгийн их утга. || $x_0 = -\frac{4}{2 \cdot (-1)} = 2$. || $y(2) = -4 + 8 + 1 = 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -11102,6 +11813,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P143" s="2" t="inlineStr">
+        <is>
+          <t>$f(4) = 3$ → $g(3) = 9$. || $g(4) = 12$ → $f(12) = 11$. || $9 - 11 = -2$.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -11177,6 +11893,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P144" s="2" t="inlineStr">
+        <is>
+          <t>Параллель шулуунууд ижил налалттай: $k = 3$. || $y = 3x + b$-д $(2;5)$: $5 = 6 + b$. || $b = -1$.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -11252,6 +11973,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P145" s="2" t="inlineStr">
+        <is>
+          <t>Дээш харсан парабол оройноосоо баруун тийш өснө. || $x_0 = -\frac{0}{2} = 0$. || Өсөх завсар: $x \ge 0$.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -11327,6 +12053,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P146" s="2" t="inlineStr">
+        <is>
+          <t>$32 = 2^5$. || $2^x = 2^5$. || $x = 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -11402,6 +12133,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P147" s="2" t="inlineStr">
+        <is>
+          <t>Ямар ч тооны тэг зэрэг 1: $a^0 = 1$. || $5^x = 5^0$. || $x = 0$.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -11477,6 +12213,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P148" s="2" t="inlineStr">
+        <is>
+          <t>$0{,}001 = \frac{1}{1000} = 10^{-3}$. || $10^x = 10^{-3}$. || $x = -3$.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -11552,6 +12293,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P149" s="2" t="inlineStr">
+        <is>
+          <t>$f(2) = 3^2 = 9$. || $f(0) = 3^0 = 1$. || $9 + 1 = 10$.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -11627,6 +12373,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P150" s="2" t="inlineStr">
+        <is>
+          <t>$8 = 2^3$, $16 = 2^4$. || $2^{3x} = 2^4$ → $3x = 4$. || $x = \frac{4}{3}$.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -11702,6 +12453,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P151" s="2" t="inlineStr">
+        <is>
+          <t>$27 = 3^3$. || $2x - 1 = 3$. || $x = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -11777,6 +12533,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P152" s="2" t="inlineStr">
+        <is>
+          <t>$\frac{1}{2} = 2^{-1}$, $8 = 2^3$. || $2^{-x} = 2^3$ → $-x = 3$. || $x = -3$.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -11852,6 +12613,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P153" s="2" t="inlineStr">
+        <is>
+          <t>Илтгэгч функц $y = a^x$: $a &gt; 1$ өснө, $0 &lt; a &lt; 1$ буурна. || $a = 0{,}5 &lt; 1$. || Буурна → $-1$.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -11927,6 +12693,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P154" s="2" t="inlineStr">
+        <is>
+          <t>$2^{x+2} = 4 \cdot 2^x$. || $4 \cdot 2^x - 2^x = 3 \cdot 2^x = 12$ → $2^x = 4$. || $x = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -12002,6 +12773,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P155" s="2" t="inlineStr">
+        <is>
+          <t>$4^x = (2^x)^2$, $t = 2^x$: $t^2 - 5t + 4 = 0$. || $t = 1$ эсвэл $t = 4$. || $2^x = 1$ → $x = 0$; $2^x = 4$ → $x = 2$.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -12077,6 +12853,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P156" s="2" t="inlineStr">
+        <is>
+          <t>$t = 5^x$: $t^2 - 6t + 5 = 0$. || $t = 1$ эсвэл $t = 5$. || $x = 0$; $x = 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -12152,6 +12933,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P157" s="2" t="inlineStr">
+        <is>
+          <t>$16 = 2^4$: $2^x &gt; 2^4$. || Суурь $2 &gt; 1$ — функц өснө, тэмдэг хадгалагдана. || $x &gt; 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -12227,6 +13013,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P158" s="2" t="inlineStr">
+        <is>
+          <t>$9 = (\tfrac{1}{3})^{-2}$: $(\tfrac{1}{3})^x \ge (\tfrac{1}{3})^{-2}$. || Суурь $&lt; 1$ — функц буурна, тэмдэг эргэнэ. || $x \le -2$.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -12302,6 +13093,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>$100 \cdot 2^t = 1600$ → $2^t = 16$. || $16 = 2^4$. || $t = 4$ цаг.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -12377,6 +13173,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>$3^? = 81$. || $3^4 = 81$. || $4$.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -12452,6 +13253,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P161" s="2" t="inlineStr">
+        <is>
+          <t>$\frac{1}{25} = 5^{-2}$. || $\log_5 5^{-2}$. || $-2$.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12527,6 +13333,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P162" s="2" t="inlineStr">
+        <is>
+          <t>$\log_a a = 1$ → $\log_7 7 = 1$. || $\log_a 1 = 0$ → $\log_7 1 = 0$. || $1 + 0 = 1$.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -12602,6 +13413,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>$0{,}01 = \frac{1}{100} = 10^{-2}$. || $\lg 10^{-2}$. || $-2$.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -12677,6 +13493,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P164" s="2" t="inlineStr">
+        <is>
+          <t>$\log_2 8 = 3$, $\log_2 4 = 2$. || $3 + 2$. || $5$ (= $\log_2 32$).</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -12752,6 +13573,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P165" s="2" t="inlineStr">
+        <is>
+          <t>$\log_3 \frac{54}{2} = \log_3 27$. || $3^3 = 27$. || $3$.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -12827,6 +13653,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P166" s="2" t="inlineStr">
+        <is>
+          <t>$\sqrt{8} = 8^{1/2}$. || $\log_a b^n = n \log_a b$: $\frac{1}{2} \log_2 8$. || $\frac{1}{2} \cdot 3 = \frac{3}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -12902,6 +13733,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P167" s="2" t="inlineStr">
+        <is>
+          <t>Тодорхойлолт: $x = 3^4$. || $3^4 = 81$. || $x = 81$.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -12977,6 +13813,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P168" s="2" t="inlineStr">
+        <is>
+          <t>Тодорхойлолт: $x^2 = 25$. || $x = \pm 5$; суурь эерэг, $\ne 1$. || $x = 5$.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -13052,6 +13893,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P169" s="2" t="inlineStr">
+        <is>
+          <t>ТМ: $x &gt; -3$ ба $x &gt; \frac{1}{2}$. Аргументууд тэнцүү: $x + 3 = 2x - 1$. || $x = 4$. || Шалгалт: $7 = 7 &gt; 0$ ✓ → $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -13127,6 +13973,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P170" s="2" t="inlineStr">
+        <is>
+          <t>Баруун тал: $\log_3 x + \log_3 2 = \log_3 2x$. || $x^2 - 8 = 2x$ → $x^2 - 2x - 8 = 0$ → $x = 4$, $x = -2$. || $x = -2$ ТМ-д орохгүй → $x = 4$.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -13202,6 +14053,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P171" s="2" t="inlineStr">
+        <is>
+          <t>Суурь солих: $\log_4 8 = \frac{\log_2 8}{\log_2 4}$. || $\frac{3}{2}$. || Хариу: $\frac{3}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -13277,6 +14133,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P172" s="2" t="inlineStr">
+        <is>
+          <t>ТМ: $x &gt; 0$. || Суурь $2 &gt; 1$: $x &lt; 2^3 = 8$. || $0 &lt; x &lt; 8$.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -13352,6 +14213,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P173" s="2" t="inlineStr">
+        <is>
+          <t>$50 = \frac{100}{2}$. || $\lg 50 = \lg 100 - \lg 2$. || $2 - a$.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -13427,6 +14293,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P174" s="2" t="inlineStr">
+        <is>
+          <t>$30°$ тусгай өнцөг. || $\cos 30° = \frac{\sqrt{3}}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -13502,6 +14373,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P175" s="2" t="inlineStr">
+        <is>
+          <t>$\operatorname{tg}\alpha = \frac{\sin\alpha}{\cos\alpha}$. || $\frac{\sqrt{3}/2}{1/2}$. || $\sqrt{3}$.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -13577,6 +14453,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P176" s="2" t="inlineStr">
+        <is>
+          <t>Тодорхойлолт: $180° = \pi$ рад.</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -13652,6 +14533,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P177" s="2" t="inlineStr">
+        <is>
+          <t>$\pi = 180°$. || $\frac{180°}{4}$. || $45°$.</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -13727,6 +14613,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P178" s="2" t="inlineStr">
+        <is>
+          <t>Үндсэн адилтгал: $\sin^2\alpha + \cos^2\alpha = 1$ ямар ч $\alpha$-д. || Шалгалт: $(\tfrac{\sqrt{2}}{2})^2 + (\tfrac{\sqrt{2}}{2})^2 = \tfrac{1}{2} + \tfrac{1}{2}$. || $1$.</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -13802,6 +14693,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P179" s="2" t="inlineStr">
+        <is>
+          <t>$\sin^2\alpha = 1 - \cos^2\alpha = 1 - \frac{25}{169} = \frac{144}{169}$. || Хурц өнцөгт $\sin\alpha &gt; 0$. || $\sin\alpha = \frac{12}{13}$.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -13877,6 +14773,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P180" s="2" t="inlineStr">
+        <is>
+          <t>$\cos\alpha = \sqrt{1 - \tfrac{9}{25}} = \frac{4}{5}$. || $\operatorname{tg}\alpha = \frac{\sin\alpha}{\cos\alpha} = \frac{3/5}{4/5}$. || $\frac{3}{4}$.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -13952,6 +14853,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P181" s="2" t="inlineStr">
+        <is>
+          <t>$150° = 180° - 30°$. || $\sin(180° - \alpha) = \sin\alpha$. || $\sin 30° = \frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -14027,6 +14933,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P182" s="2" t="inlineStr">
+        <is>
+          <t>$120° = 180° - 60°$. || $\cos(180° - \alpha) = -\cos\alpha$. || $-\cos 60° = -\frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -14102,6 +15013,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P183" s="2" t="inlineStr">
+        <is>
+          <t>Нэгж тойрог дээр $\cos x = 0$ — $x$ координат нь 0 цэгүүд. || Дээд цэг $\frac{\pi}{2}$, доод цэг $\frac{3\pi}{2}$. || $x = \frac{\pi}{2}$; $x = \frac{3\pi}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -14177,6 +15093,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P184" s="2" t="inlineStr">
+        <is>
+          <t>$\sin x = \frac{1}{2}$. || I мөчлөг: $\frac{\pi}{6}$; II мөчлөг: $\pi - \frac{\pi}{6} = \frac{5\pi}{6}$. || $x = \frac{\pi}{6}$; $x = \frac{5\pi}{6}$.</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -14252,6 +15173,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P185" s="2" t="inlineStr">
+        <is>
+          <t>$\operatorname{ctg}\alpha = \frac{\cos\alpha}{\sin\alpha}$. || $\sin\alpha \cdot \frac{\cos\alpha}{\sin\alpha}$. || $\cos\alpha$.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -14327,6 +15253,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P186" s="2" t="inlineStr">
+        <is>
+          <t>$(1-s)(1+s) = 1 - s^2$. || $1 - \sin^2\alpha$. || $= \cos^2\alpha$ (үндсэн адилтгал).</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -14402,6 +15333,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P187" s="2" t="inlineStr">
+        <is>
+          <t>$390° = 360° + 30°$. || Үе $360°$: $\sin 390° = \sin 30°$. || $\frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -14477,6 +15413,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P188" s="2" t="inlineStr">
+        <is>
+          <t>Үр дүн 2: сүлд, тоо. || Таатай нь 1. || $P = \frac{1}{2}$.</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -14552,6 +15493,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P189" s="2" t="inlineStr">
+        <is>
+          <t>5-аас их тоо шоон дээр: зөвхөн 6. || Таатай 1, нийт 6. || $P = \frac{1}{6}$.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -14627,6 +15573,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P190" s="2" t="inlineStr">
+        <is>
+          <t>3-т хуваагдах: 3, 6, 9 — 3 ширхэг. || Нийт 10. || $P = \frac{3}{10}$.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -14702,6 +15653,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P191" s="2" t="inlineStr">
+        <is>
+          <t>$P(A) + P(\bar A) = 1$. || $P(\bar A) = 1 - 0{,}3$. || $0{,}7$.</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -14777,6 +15733,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P192" s="2" t="inlineStr">
+        <is>
+          <t>Нийт $4 + 6 = 10$. || Таатай (хар) 6. || $\frac{6}{10} = \frac{3}{5}$.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -14852,6 +15813,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P193" s="2" t="inlineStr">
+        <is>
+          <t>Эхний байранд 4 сонголт, дараа нь 3, 2, 1. || $4! = 4 \cdot 3 \cdot 2 \cdot 1$. || $24$.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -14927,6 +15893,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P194" s="2" t="inlineStr">
+        <is>
+          <t>Албан тушаал өөр тул дараалал чухал (байрлуулал). || Ахлагч 6 сонголт, орлогч үлдсэн 5. || $6 \cdot 5 = 30$.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -15002,6 +15973,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P195" s="2" t="inlineStr">
+        <is>
+          <t>Дараалал чухал биш → хэсэглэл. || $C_5^2 = \frac{5 \cdot 4}{2}$. || $10$.</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -15077,6 +16053,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P196" s="2" t="inlineStr">
+        <is>
+          <t>Үржүүлэх дүрэм: цамц бүрт 4 өмд тохирно. || $3 \cdot 4$. || $12$.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -15152,6 +16133,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P197" s="2" t="inlineStr">
+        <is>
+          <t>Хоёр шоо бие даасан. || $P = P_1 \cdot P_2 = \frac{1}{6} \cdot \frac{1}{6}$. || $\frac{1}{36}$.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -15227,6 +16213,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P198" s="2" t="inlineStr">
+        <is>
+          <t>Нийт 36. Нийлбэр 10: (4,6),(5,5),(6,4); 11: (5,6),(6,5); 12: (6,6). || Таатай $3 + 2 + 1 = 6$. || $\frac{6}{36} = \frac{1}{6}$.</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -15302,6 +16293,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P199" s="2" t="inlineStr">
+        <is>
+          <t>Тэгш: {2, 4, 6}; 3-т хуваагдах: {3, 6}. || Нэгдэл: {2, 3, 4, 6} — 6-г нэг л удаа тоолно. || $\frac{4}{6} = \frac{2}{3}$.</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -15377,6 +16373,11 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P200" s="2" t="inlineStr">
+        <is>
+          <t>Сүлд 4 хаялтын алинд нь ч буух боломжтой: $C_4^1 = 4$. || Тодорхой нэг дараалал: $(\tfrac{1}{2})^4 = \frac{1}{16}$. || $4 \cdot \frac{1}{16} = \frac{1}{4}$.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -15452,9 +16453,14 @@
           <t>OK</t>
         </is>
       </c>
+      <c r="P201" s="2" t="inlineStr">
+        <is>
+          <t>Эхний бөмбөг улаан: $\frac{3}{5}$. || Буцаагаагүй: үлдсэн 4-өөс улаан 2 → $\frac{2}{4}$. || $\frac{3}{5} \cdot \frac{2}{4} = \frac{3}{10}$.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O201"/>
+  <autoFilter ref="A1:P201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>